<commit_message>
Correct packing-slip reads from the page images.
The AQPC invoice and PO boxes are readable by eye. None of those slips match a live AP bill yet, so they stay off. McMaster PO 59235 qty 3 was already on bill 10144.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/packing-slips-catchup-2026-10-05.xlsx
+++ b/runs/packing-slips-catchup-2026-10-05.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Packing slips" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Packing slips'!$A$1:$J$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Packing slips'!$A$1:$K$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -446,19 +446,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="42" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="46" customWidth="1" min="9" max="9"/>
-    <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -512,6 +513,11 @@
           <t>Why stuck</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Read by eye</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -557,7 +563,12 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>No matching bill/PO yet. Readable JAR-TEX form for PO 59244 (doc 58673). No JAR-TEX / Billmark bill on that PO. No sanctioned attach-to-PO path.</t>
+          <t>No matching bill yet. Eye read is clear. No JAR-TEX bill for invoice 58673 or PO 59244.</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>JAR-TEX Industries (dba Billmark Plating); PO 59244; invoice/slip 58673; qty 5, 3, and 1</t>
         </is>
       </c>
     </row>
@@ -605,7 +616,12 @@
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>No matching bill/PO yet. Crosslink packing slip 5511, PO 59258, qty 3. No Crosslink bill on that PO.</t>
+          <t>No matching bill yet. Eye read is clear. No Crosslink bill for slip 5511 or PO 59258.</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Crosslink Powder Coating; PO 59258; invoice/slip 5511; qty 3 of 1020249-1</t>
         </is>
       </c>
     </row>
@@ -637,12 +653,12 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>77436</t>
+          <t>11057</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>1 each on lines 1-8 (6000880-001 / related basket parts)</t>
+          <t>1 each on 8 lines (packlist 77436)</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -653,7 +669,12 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>No matching bill/PO yet. AQPC packlist 77436, PO 59335. No AQPC bill on that PO.</t>
+          <t>No matching bill yet. Eye read: AQPC invoice 11057, PO 59335, qty 1 per line. No AQPC bill with that invoice or PO.</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating; PO 59335; invoice/slip 11057; qty 1 each, 8 lines</t>
         </is>
       </c>
     </row>
@@ -685,12 +706,12 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>77361</t>
+          <t>11056</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>1 of A060R267; 4 of A059J397; 1 of 70040164; 1 of A059J396</t>
+          <t>1 of A060R267; 4 of A059J397; 1 of 70040164; 1 of A059J396 (packlist 77361)</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -701,7 +722,12 @@
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>No matching bill/PO yet. AQPC packlist 77361, PO 59331. No AQPC bill on that PO.</t>
+          <t>No matching bill yet. Eye read: AQPC invoice 11056, PO 59331. The letterhead page of the same invoice shows A059J397 qty 1, this packlist shows qty 4. No AQPC bill to attach to either page.</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating; PO 59331; invoice/slip 11056; qty 1, 4, 1, 1</t>
         </is>
       </c>
     </row>
@@ -733,12 +759,12 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>77359</t>
+          <t>11055</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>1 of M4.9-2065; 1 of M4.9-2066; 1 of M4.9-2067; 3 of M4.2A</t>
+          <t>1+1+1 of M4.9 parts; 3 of M4.2A (packlist 77359)</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -749,7 +775,12 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>No matching bill/PO yet. AQPC packlist 77359, PO 59330. No AQPC bill on that PO.</t>
+          <t>No matching bill yet. Eye read: AQPC invoice 11055, PO 59330. No AQPC bill with that invoice or PO.</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating; PO 59330; invoice/slip 11055; qty 1, 1, 1, and 3</t>
         </is>
       </c>
     </row>
@@ -781,12 +812,12 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>77362</t>
+          <t>11058</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>20 of 5001914-003</t>
+          <t>20 of 5001914-003 (packlist 77362)</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -797,7 +828,12 @@
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>No matching bill/PO yet. AQPC packlist 77362, PO 59333 line 01, qty 20. No AQPC bill on that PO.</t>
+          <t>No matching bill yet. Eye read: AQPC invoice 11058, PO 59333, qty 20. No AQPC bill with that invoice or PO.</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating; PO 59333; invoice/slip 11058; qty 20</t>
         </is>
       </c>
     </row>
@@ -834,7 +870,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>48 shipped of KANNON-ME26-1951 (ordered 48)</t>
+          <t>48 of KANNON-ME26-1951</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -845,7 +881,12 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>No matching bill/PO yet. Legacy Wire shipment S-SHPT103393, PO 59322, qty 48. No Legacy Wire bill on that PO. Page 2 of this PDF is a different shipment.</t>
+          <t>No matching bill yet. Eye read: Legacy Wire shipment S-SHPT103393, order S-ORD102051, PO 59322, qty 48. No Legacy Wire bill on that PO.</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Legacy Wire Products; PO 59322; invoice/slip S-SHPT103393 / S-ORD102051; qty 48</t>
         </is>
       </c>
     </row>
@@ -882,7 +923,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>27 shipped of KANNON-ME26-1951 (ordered 27)</t>
+          <t>27 of KANNON-ME26-1951</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -893,7 +934,12 @@
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>No matching bill/PO yet. Legacy Wire shipment S-SHPT103392, PO 59334, qty 27. No Legacy Wire bill on that PO.</t>
+          <t>No matching bill yet. Eye read: Legacy Wire shipment S-SHPT103392, order S-ORD102050, PO 59334, qty 27. No Legacy Wire bill on that PO.</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Legacy Wire Products; PO 59334; invoice/slip S-SHPT103392 / S-ORD102050; qty 27</t>
         </is>
       </c>
     </row>
@@ -926,7 +972,7 @@
       <c r="F10" s="2" t="inlineStr"/>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>90 required of 18160536-001 (order quantity, not a shipped qty)</t>
+          <t>90 ordered of 18160536-001</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -937,7 +983,12 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Not a packing slip. The scan is Kannon purchase order 59337 to JARTEX (qty required 90). Left off.</t>
+          <t>Not a packing slip. Eye read is a Kannon purchase order 59337 to JARTEX, qty required 90. Left off.</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>JARTEX Industries (purchase order, not a packing slip); PO 59337; invoice/slip —; qty 90 ordered</t>
         </is>
       </c>
     </row>
@@ -962,11 +1013,19 @@
           <t>American Quality Powder Coating</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>59331</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>11056</t>
+        </is>
+      </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>1 of A060R267; 1 of A059J397; 1 of 70040164; 1 of A059J396</t>
+          <t>1 each of A060R267, A059J397, 70040164, A059J396</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -977,7 +1036,12 @@
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Unreadable match key. AQPC packing slip with quantities, but no PO number and no invoice/packlist number on the page.</t>
+          <t>No matching bill yet. Eye read: AQPC invoice 11056, PO 59331, qty 1 each. The formal packlist for the same invoice shows A059J397 qty 4. No AQPC bill to attach to either page.</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating; PO 59331; invoice/slip 11056; qty 1, 1, 1, 1</t>
         </is>
       </c>
     </row>
@@ -1002,8 +1066,16 @@
           <t>American Quality Powder Coating</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>59330</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>11055</t>
+        </is>
+      </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
           <t>3 of KAN-M4.9; 3 of KAN-M4.2</t>
@@ -1017,7 +1089,12 @@
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Unreadable match key. AQPC packing slip with quantities, but no PO number and no invoice/packlist number on the page.</t>
+          <t>No matching bill yet. Eye read: AQPC invoice 11055, PO 59330, qty 3 and 3. Consistent with the itemized packlist (1+1+1 and 3). No AQPC bill with that invoice or PO.</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating; PO 59330; invoice/slip 11055; qty 3 and 3</t>
         </is>
       </c>
     </row>
@@ -1049,12 +1126,12 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>77391</t>
+          <t>6-175802</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>6 of 12519-2</t>
+          <t>6 of 12519-2 (packlist 77391)</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
@@ -1065,7 +1142,12 @@
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>No matching bill/PO yet. Arrow packlist 77391, PO 59321, qty 6. No Arrow bill on that PO.</t>
+          <t>No matching bill yet. Eye read: Arrow invoice 6-175802, PO 59321, qty 6. No Arrow bill with that invoice or PO.</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Arrow Plating; PO 59321; invoice/slip 6-175802; qty 6 of 12519-2</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1184,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>quantity column not readable (parts 1020249-1 and 1020249-4; leading digits are line numbers)</t>
+          <t>1 of 1020249-1; 2 of 1020249-4</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
@@ -1113,7 +1195,12 @@
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Unreadable quantity. Crosslink slip 5493 names PO 59258, but the shipped quantity did not read cleanly. Left off.</t>
+          <t>No matching bill yet. Eye read: Crosslink slip 5493, PO 59258, qty 1 and 2. No Crosslink bill for that slip or PO.</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Crosslink Powder Coating; PO 59258; invoice/slip 5493; qty 1 and 2</t>
         </is>
       </c>
     </row>
@@ -1138,8 +1225,16 @@
           <t>American Quality Powder Coating</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>59311</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>11053</t>
+        </is>
+      </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
           <t>12 of AMT-F1508</t>
@@ -1153,7 +1248,12 @@
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Unreadable match key. AQPC packing slip, qty 12, no PO number and no invoice/packlist number.</t>
+          <t>No matching bill yet. Eye read: AQPC invoice 11053, PO 59311, date 09/30/2026, qty 12. No AQPC bill with invoice 11053 or PO 59311. KANNON/CDM invoice 59311 (id 1298) is a different vendor.</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating; PO 59311; invoice/slip 11053; qty 12 of AMT-F1508</t>
         </is>
       </c>
     </row>
@@ -1178,8 +1278,16 @@
           <t>American Quality Powder Coating</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>59315</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>11052</t>
+        </is>
+      </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
           <t>15 of A060P934</t>
@@ -1193,7 +1301,12 @@
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Unreadable match key. AQPC packing slip, qty 15, no PO number and no invoice/packlist number.</t>
+          <t>No matching bill yet. Eye read: AQPC invoice 11052, PO 59315, qty 15. No AQPC bill with that invoice or PO.</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating; PO 59315; invoice/slip 11052; qty 15 of A060P934</t>
         </is>
       </c>
     </row>
@@ -1218,11 +1331,19 @@
           <t>American Quality Powder Coating</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>59312</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>11050</t>
+        </is>
+      </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>quantity not separated cleanly from RAL 9016 (part 5003557-001, SO34831)</t>
+          <t>5 of 5003557-001</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -1233,7 +1354,12 @@
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Unreadable match key. AQPC packing slip with no PO number and no reliable quantity.</t>
+          <t>No matching bill yet. Eye read: AQPC invoice 11050, PO 59312, qty 5. No AQPC bill with that invoice or PO.</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating; PO 59312; invoice/slip 11050; qty 5 of 5003557-001</t>
         </is>
       </c>
     </row>
@@ -1258,11 +1384,19 @@
           <t>American Quality Powder Coating</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>59314</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>11049</t>
+        </is>
+      </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>quantity not separated cleanly from RAL 9016 (part 5003557-001, SO34826)</t>
+          <t>10 of 5003557-001</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
@@ -1273,7 +1407,12 @@
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Unreadable match key. AQPC packing slip with no PO number and no reliable quantity.</t>
+          <t>No matching bill yet. Eye read: AQPC invoice 11049, PO 59314, qty 10. No AQPC bill with that invoice or PO.</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating; PO 59314; invoice/slip 11049; qty 10 of 5003557-001</t>
         </is>
       </c>
     </row>
@@ -1298,8 +1437,16 @@
           <t>American Quality Powder Coating</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>59313</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>11051</t>
+        </is>
+      </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
           <t>12 of 55700014</t>
@@ -1313,7 +1460,12 @@
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Unreadable match key. AQPC packing slip, qty 12, no PO number and no invoice/packlist number.</t>
+          <t>No matching bill yet. Eye read: AQPC invoice 11051, PO 59313, qty 12. No AQPC bill with that invoice or PO.</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating; PO 59313; invoice/slip 11051; qty 12 of 55700014</t>
         </is>
       </c>
     </row>
@@ -1338,8 +1490,16 @@
           <t>American Quality Powder Coating</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>59298</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>11048</t>
+        </is>
+      </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
           <t>18 of A074A683; 18 of A074A682; 10 of 5001914; 1 of 80341994</t>
@@ -1353,7 +1513,12 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Unreadable match key. AQPC packing slip with quantities, but no PO number and no invoice/packlist number.</t>
+          <t>No matching bill yet. Eye read: AQPC invoice 11048, PO 59298, those four quantities. No AQPC bill with that invoice or PO.</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating; PO 59298; invoice/slip 11048; qty 18, 18, 10, 1</t>
         </is>
       </c>
     </row>
@@ -1390,7 +1555,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>quantity not readable (part 1020249-1)</t>
+          <t>1 of 1020249-1</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -1401,7 +1566,12 @@
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Unreadable quantity. Crosslink slip 5499 names PO 59225, but the shipped quantity did not read. Left off. Invoice 59225 (id 1291) is vendor KANNON/CDM, not Crosslink.</t>
+          <t>No matching bill yet. Eye read: Crosslink slip 5499, PO 59225, qty 1. No Crosslink bill for that slip or PO.</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Crosslink Powder Coating; PO 59225; invoice/slip 5499; qty 1 of 1020249-1</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1619,12 @@
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>No matching bill/PO yet. Arrow shipping ticket order 179924, PO 58743, qty 350. No Arrow bill on that PO.</t>
+          <t>No matching bill yet. Eye read: Arrow order 179924, PO 58743, qty 350. No Arrow bill on that PO.</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Arrow Plating; PO 58743; invoice/slip 179924; qty 350 of 1007092-1</t>
         </is>
       </c>
     </row>
@@ -1474,11 +1649,19 @@
           <t>American Quality Powder Coating</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr"/>
-      <c r="F23" s="2" t="inlineStr"/>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>59302</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>11041</t>
+        </is>
+      </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>5 of 6001232; 5 and 5 of 5003753; 15 of 5003741; 5 of 5003750-002; 5 of 5003750 (SO34645)</t>
+          <t>5, 5, 5, 15, 5, 5 (SO34645 basket set)</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
@@ -1489,7 +1672,12 @@
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Unreadable match key. AQPC packing slip with quantities, but no PO number and no invoice/packlist number.</t>
+          <t>No matching bill yet. Eye read: AQPC invoice 11041, PO 59302. No AQPC bill with that invoice or PO.</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating; PO 59302; invoice/slip 11041; qty 5, 5, 5, 15, 5, 5</t>
         </is>
       </c>
     </row>
@@ -1514,8 +1702,16 @@
           <t>American Quality Powder Coating</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>59287</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>11042</t>
+        </is>
+      </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
           <t>5 of 5003522-001</t>
@@ -1529,7 +1725,12 @@
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Unreadable match key. AQPC packing slip, qty 5, no PO number and no invoice/packlist number.</t>
+          <t>No matching bill yet. Eye read: AQPC invoice 11042, PO 59287, qty 5. No AQPC bill with that invoice or PO.</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating; PO 59287; invoice/slip 11042; qty 5 of 5003522-001</t>
         </is>
       </c>
     </row>
@@ -1554,11 +1755,19 @@
           <t>American Quality Powder Coating</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr"/>
-      <c r="F25" s="2" t="inlineStr"/>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>59303</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>11043</t>
+        </is>
+      </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>1 of 6001232; 1 and 1 of 5003753; 3 of 5003741; 1 of 5003750-002; 1 of 5003750 (P089476)</t>
+          <t>1, 1, 1, 3, 1, 1 (P089476 basket set)</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
@@ -1569,7 +1778,12 @@
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Unreadable match key. AQPC packing slip with quantities, but no PO number and no invoice/packlist number.</t>
+          <t>No matching bill yet. Eye read: AQPC invoice 11043, PO 59303. No AQPC bill with that invoice or PO.</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating; PO 59303; invoice/slip 11043; qty 1, 1, 1, 3, 1, 1</t>
         </is>
       </c>
     </row>
@@ -1594,8 +1808,16 @@
           <t>American Quality Powder Coating</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>59274</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>11044</t>
+        </is>
+      </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
           <t>250 of KAN-MD04</t>
@@ -1609,7 +1831,12 @@
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Unreadable match key. AQPC packing slip, qty 250, no PO number and no invoice/packlist number.</t>
+          <t>No matching bill yet. Eye read: AQPC invoice 11044, PO 59274, qty 250. No AQPC bill with invoice 11044 or PO 59274. A different slip (invoice 11054, packlist 77271) is also qty 250 on PO 59274.</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating; PO 59274; invoice/slip 11044; qty 250 of KAN-MD04</t>
         </is>
       </c>
     </row>
@@ -1641,12 +1868,12 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>77329</t>
+          <t>6-175800</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>26 of 5003004-001</t>
+          <t>26 of 5003004-001 (packlist 77329)</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
@@ -1657,7 +1884,12 @@
       <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>No matching bill/PO yet. Arrow packlist 77329, PO 59310, qty 26. No Arrow bill on that PO.</t>
+          <t>No matching bill yet. Eye read: Arrow invoice 6-175800, PO 59310, qty 26. No Arrow bill with that invoice or PO.</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Arrow Plating; PO 59310; invoice/slip 6-175800; qty 26 of 5003004-001</t>
         </is>
       </c>
     </row>
@@ -1689,12 +1921,12 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>77326</t>
+          <t>6-175797</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>2 of 33214-1</t>
+          <t>2 of 33214-1 (packlist 77326)</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
@@ -1705,7 +1937,12 @@
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>No matching bill/PO yet. Arrow packlist 77326, PO 59307, qty 2. No Arrow bill on that PO.</t>
+          <t>No matching bill yet. Eye read: Arrow invoice 6-175797, PO 59307, qty 2. No Arrow bill with that invoice or PO.</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Arrow Plating; PO 59307; invoice/slip 6-175797; qty 2 of 33214-1</t>
         </is>
       </c>
     </row>
@@ -1737,12 +1974,12 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>77328</t>
+          <t>6-175799</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>100 of 7766-1</t>
+          <t>100 of 7766-1 (packlist 77328)</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
@@ -1753,7 +1990,12 @@
       <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>No matching bill/PO yet. Arrow packlist 77328, PO 59309, qty 100. No Arrow bill on that PO.</t>
+          <t>No matching bill yet. Eye read: Arrow invoice 6-175799, PO 59309, qty 100. No Arrow bill with that invoice or PO.</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Arrow Plating; PO 59309; invoice/slip 6-175799; qty 100 of 7766-1</t>
         </is>
       </c>
     </row>
@@ -1785,12 +2027,12 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>77327</t>
+          <t>6-175798</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>300 of 7766-1</t>
+          <t>300 of 7766-1 (packlist 77327)</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
@@ -1801,7 +2043,12 @@
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>No matching bill/PO yet. Arrow packlist 77327, PO 59308, qty 300. No Arrow bill on that PO.</t>
+          <t>No matching bill yet. Eye read: Arrow invoice 6-175798, PO 59308, qty 300. No Arrow bill with that invoice or PO.</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Arrow Plating; PO 59308; invoice/slip 6-175798; qty 300 of 7766-1</t>
         </is>
       </c>
     </row>
@@ -1821,7 +2068,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr"/>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating</t>
+        </is>
+      </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
           <t>59314</t>
@@ -1829,12 +2080,12 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>77332</t>
+          <t>11049</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>quantity not readable (part 5003557-001; '10 WHITE' reads as the finish, not a shipped qty)</t>
+          <t>10 of 5003557-001 (packlist 77332)</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
@@ -1845,7 +2096,12 @@
       <c r="I31" s="2" t="inlineStr"/>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>Unreadable. Packlist 77332 names PO 59314, but the vendor name is not on the page (both addresses are Kannon) and the shipped quantity did not read.</t>
+          <t>No matching bill yet. Eye read: AQPC invoice 11049, PO 59314, qty 10. Same invoice as the letterhead page. No AQPC bill with that invoice or PO.</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating; PO 59314; invoice/slip 11049; qty 10 of 5003557-001</t>
         </is>
       </c>
     </row>
@@ -1877,12 +2133,12 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>77331</t>
+          <t>11050</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>5 of 5003557-001</t>
+          <t>5 of 5003557-001 (packlist 77331)</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
@@ -1893,7 +2149,12 @@
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>No matching bill/PO yet. AQPC packlist 77331, PO 59312, qty 5. No AQPC bill on that PO. Invoice 59312 (id 1299) is vendor KANNON/CDM, not AQPC.</t>
+          <t>No matching bill yet. Eye read: AQPC invoice 11050, PO 59312, qty 5. Same invoice as the letterhead page. No AQPC bill with that invoice or PO.</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating; PO 59312; invoice/slip 11050; qty 5 of 5003557-001</t>
         </is>
       </c>
     </row>
@@ -1913,7 +2174,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr"/>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating</t>
+        </is>
+      </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
           <t>59315</t>
@@ -1921,12 +2186,12 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>77333</t>
+          <t>11052</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>15 of A060P934</t>
+          <t>15 of A060P934 (packlist 77333)</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -1937,7 +2202,12 @@
       <c r="I33" s="2" t="inlineStr"/>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>Unreadable vendor. Packlist 77333, PO 59315, qty 15, but the vendor name is not on the page (addresses are Kannon only). Left off.</t>
+          <t>No matching bill yet. Eye read: AQPC invoice 11052, PO 59315, qty 15. Same invoice as the letterhead page. No AQPC bill with that invoice or PO.</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating; PO 59315; invoice/slip 11052; qty 15 of A060P934</t>
         </is>
       </c>
     </row>
@@ -1957,7 +2227,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating</t>
+        </is>
+      </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
           <t>59311</t>
@@ -1965,12 +2239,12 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>77330</t>
+          <t>11053</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>12 of F1508</t>
+          <t>12 of F1508 (packlist 77330)</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
@@ -1981,7 +2255,12 @@
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>Unreadable vendor. Packlist 77330, PO 59311, qty 12, but the vendor name is not on the page. Invoice 59311 (id 1298) is vendor KANNON/CDM, which does not match a blank vendor. Left off.</t>
+          <t>No matching bill yet. Eye read: AQPC invoice 11053, PO 59311, qty 12. Same invoice Kyle checked on the letterhead page. No AQPC bill with invoice 11053 or PO 59311.</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating; PO 59311; invoice/slip 11053; qty 12 of F1508</t>
         </is>
       </c>
     </row>
@@ -2013,12 +2292,12 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>77341 or 77344 (OCR disagree)</t>
+          <t>11048</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>line quantities disagreed across OCR passes (18 vs 48 vs 6 on the second engine support)</t>
+          <t>18, 18, 10, 1 (packlist 77341)</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
@@ -2029,7 +2308,12 @@
       <c r="I35" s="2" t="inlineStr"/>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>Unreadable quantity. AQPC packlist on PO 59298, but shipped quantities were not stable across rotations/PSM and the packlist number read as both 77341 and 77344. Left off.</t>
+          <t>No matching bill yet. Eye read: AQPC invoice 11048, PO 59298, qty 18, 18, 10, and 1. Same invoice as the letterhead page. No AQPC bill with that invoice or PO.</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating; PO 59298; invoice/slip 11048; qty 18, 18, 10, 1</t>
         </is>
       </c>
     </row>
@@ -2077,7 +2361,12 @@
       <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>No matching bill/PO yet. Arrow shipping ticket order 179880, PO 58722, qty 100. No Arrow bill on that PO.</t>
+          <t>No matching bill yet. Eye read: Arrow order 179880, PO 58722, qty 100. No Arrow bill on that PO.</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>Arrow Plating; PO 58722; invoice/slip 179880; qty 100 of 11772-1</t>
         </is>
       </c>
     </row>
@@ -2125,7 +2414,12 @@
       <c r="I37" s="2" t="inlineStr"/>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>No matching bill/PO yet. Arrow shipping ticket order 180005, PO 58882, qty 50. No Arrow bill on that PO.</t>
+          <t>No matching bill yet. Eye read: Arrow order 180005, PO 58882, qty 50. No Arrow bill on that PO.</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Arrow Plating; PO 58882; invoice/slip 180005; qty 50 of 11772-1</t>
         </is>
       </c>
     </row>
@@ -2157,12 +2451,12 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>77271</t>
+          <t>11054</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>250 of MD04-1661 (marked page 4 of the packlist)</t>
+          <t>250 of MD04-1661 (packlist 77271, marked page 4)</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
@@ -2173,7 +2467,12 @@
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>No matching bill/PO yet. AQPC packlist 77271 page 4, PO 59274, qty 250. No AQPC bill on that PO. Invoice 59274 (id 286) is vendor KANNON/CDM, not AQPC.</t>
+          <t>No matching bill yet. Eye read: AQPC invoice 11054, PO 59274, qty 250. No AQPC bill with invoice 11054 or PO 59274.</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>American Quality Powder Coating; PO 59274; invoice/slip 11054; qty 250 of MD04-1661</t>
         </is>
       </c>
     </row>
@@ -2210,18 +2509,23 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>shipped quantity did not read (part 91306A416, packs of 10; bill line is qty 3)</t>
-        </is>
-      </c>
-      <c r="H39" s="3" t="inlineStr">
-        <is>
-          <t>Stuck</t>
-        </is>
-      </c>
-      <c r="I39" s="2" t="inlineStr"/>
-      <c r="J39" s="2" t="inlineStr">
-        <is>
-          <t>Unreadable quantity. McMaster PO 59235 matches only bill 10144 (vendor invoice 72087570), whose line is qty 3 of 91306A416. The slip's shipped quantity did not OCR cleanly, so this run did not attach. A prior file packing-slip-59235-page 1.pdf is already on that bill; it was not removed or replaced.</t>
+          <t>3 shipped of 91306A416 (ordered 3)</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>Attached</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>KIMCO bill 10144, vendor invoice 72087570 (already on header as packing-slip-59235-page 1.pdf; not re-uploaded)</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr"/>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>McMaster-Carr; PO 59235; invoice/slip 5756929-01; qty ordered 3, shipped 3 of 91306A416</t>
         </is>
       </c>
     </row>
@@ -2269,7 +2573,12 @@
       <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>No matching bill/PO yet. Slip vendor is McMaster, PO 58221, qty 24. The only live bill on PO 58221 is AQPC invoice 10655 (id 8827). Vendor does not match, so it was left off.</t>
+          <t>No matching bill yet. Eye read: McMaster PO 58221, qty 24. The only live bill on PO 58221 is AQPC invoice 10655 (id 8827). Vendor does not match.</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>McMaster-Carr; PO 58221; invoice/slip 5687917-01; qty ordered 24, shipped 24 of 4082715</t>
         </is>
       </c>
     </row>
@@ -2320,6 +2629,11 @@
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr"/>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>McMaster-Carr; PO 59191; invoice/slip 5539373-01; qty ordered 40, shipped 40 of 91247A860</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2354,7 +2668,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>line 4 (93320A385) shipped 1; other lines on the slip are not on this bill</t>
+          <t>line 4 shipped 1 of 93320A385 (ordered 2); lines 1-3 also printed</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
@@ -2368,6 +2682,11 @@
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>McMaster-Carr; PO 59224; invoice/slip 5765761-01; qty line 4 ordered 2, shipped 1</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2402,7 +2721,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>line 4 shipped 1 (Chicago shipment), plus lines 1-3</t>
+          <t>line 4 shipped 1 of 93320A385; lines 1-3 shipped 6, 1, and 1</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
@@ -2413,7 +2732,12 @@
       <c r="I43" s="2" t="inlineStr"/>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>Qty conflict. Bill 10142 (vendor invoice 72094446) is PO 59224 line 04 qty 1, already matched to packing list 5765761-01. This second list (5765761-02) also shows line 4 shipped 1, which would put shipped qty 2 on a qty-1 bill. Left off. A prior file packing-slip-59224-page 2.pdf is already on the bill; it was not removed.</t>
+          <t>Qty conflict. Eye read: McMaster list 5765761-02, PO 59224, line 4 shipped 1. Bill 10142 is PO line 04 qty 1 and already has list 5765761-01 (also line 4 shipped 1). Putting this second shipment on that bill would show shipped qty 2 against qty 1. Left off. A prior file packing-slip-59224-page 2.pdf is already on the bill and was not removed.</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>McMaster-Carr; PO 59224; invoice/slip 5765761-02; qty line 4 ordered 2, shipped 1; lines 1-3 shipped 6, 1, 1</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2762,11 @@
           <t>McMaster-Carr</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>59149</t>
+        </is>
+      </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
           <t>5680403-07</t>
@@ -2446,7 +2774,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>40 shipped of 91247A860 (ordered 40)</t>
+          <t>40 shipped of 91247A866 (ordered 40)</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
@@ -2457,12 +2785,17 @@
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>Unreadable PO. McMaster packing list 5680403-07, qty 40, but the purchase-order number did not read. Left off rather than guess a PO.</t>
+          <t>No matching bill yet. Eye read: McMaster PO 59149, order 5680403-07, qty 40 of 91247A866. No McMaster bill on PO 59149.</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>McMaster-Carr; PO 59149; invoice/slip 5680403-07; qty ordered 40, shipped 40 of 91247A866</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J44"/>
+  <autoFilter ref="A1:K44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Correct packing-slip workbook rows from header and quantity crops.
Each receiving page was re-read from a binarized crop of the invoice, date, and PO box and of the quantity column, and the workbook row for that file and page was set to those printed values.

Co-authored-by: beave89atm <beave89atm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/runs/packing-slips-catchup-2026-10-05.xlsx
+++ b/runs/packing-slips-catchup-2026-10-05.xlsx
@@ -563,12 +563,12 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read is clear. No JAR-TEX bill for invoice 58673 or PO 59244.</t>
+          <t>No matching bill yet. Crop read: JAR-TEX slip 58673, PO 59244, date Sep 21, 2026, those three quantities. No JAR-TEX bill for that slip or PO.</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>JAR-TEX Industries (dba Billmark Plating); PO 59244; invoice/slip 58673; qty 5, 3, and 1</t>
+          <t>JAR-TEX Industries (dba Billmark Plating); PO 59244; slip 58673; date Sep 21, 2026; qty 5, 3, and 1</t>
         </is>
       </c>
     </row>
@@ -616,12 +616,12 @@
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read is clear. No Crosslink bill for slip 5511 or PO 59258.</t>
+          <t>No matching bill yet. Crop read: Crosslink slip 5511, PO 59258, date Thu Oct 1 2026, qty 3. No Crosslink bill for that slip or PO.</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Crosslink Powder Coating; PO 59258; invoice/slip 5511; qty 3 of 1020249-1</t>
+          <t>Crosslink Powder Coating; PO 59258; slip 5511; date Oct 1, 2026; qty 3 of 1020249-1</t>
         </is>
       </c>
     </row>
@@ -653,12 +653,12 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>11057</t>
+          <t>77436</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>1 each on 8 lines (packlist 77436)</t>
+          <t>1 each on 8 lines of 6000880-001 (packlist 77436)</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -669,12 +669,12 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: AQPC invoice 11057, PO 59335, qty 1 per line. No AQPC bill with that invoice or PO.</t>
+          <t>No matching bill yet. This page is a Kannon packlist, not an AQPC letterhead. Packlist 77436, ship date 10/1/2026, PO 59335, qty 1 on eight lines. No Invoice no. is printed. No AQPC bill on PO 59335.</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>American Quality Powder Coating; PO 59335; invoice/slip 11057; qty 1 each, 8 lines</t>
+          <t>American Quality Powder Coating; PO 59335; packlist 77436; ship date 10/1/2026; qty 1 each, 8 lines; no invoice number printed</t>
         </is>
       </c>
     </row>
@@ -706,12 +706,12 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>11056</t>
+          <t>77361</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>1 of A060R267; 4 of A059J397; 1 of 70040164; 1 of A059J396 (packlist 77361)</t>
+          <t>1 of A060R267; 4 of A059J397; 1 of 70040164; 1 of A059J396</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -722,12 +722,12 @@
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: AQPC invoice 11056, PO 59331. The letterhead page of the same invoice shows A059J397 qty 1, this packlist shows qty 4. No AQPC bill to attach to either page.</t>
+          <t>No matching bill yet. Kannon packlist 77361, ship date 9/30/2026, PO 59331, those quantities. No Invoice no. is printed on this page. No AQPC bill on PO 59331.</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>American Quality Powder Coating; PO 59331; invoice/slip 11056; qty 1, 4, 1, 1</t>
+          <t>American Quality Powder Coating; PO 59331; packlist 77361; ship date 9/30/2026; qty 1, 4, 1, 1; no invoice number printed</t>
         </is>
       </c>
     </row>
@@ -759,12 +759,12 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>11055</t>
+          <t>77359</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>1+1+1 of M4.9 parts; 3 of M4.2A (packlist 77359)</t>
+          <t>1 of M4.9-2065; 1 of M4.9-2066; 1 of M4.9-2067; 3 of M4.2A</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -775,12 +775,12 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: AQPC invoice 11055, PO 59330. No AQPC bill with that invoice or PO.</t>
+          <t>No matching bill yet. Kannon packlist 77359, ship date 9/30/2026, PO 59330, those quantities. No Invoice no. is printed. No AQPC bill on PO 59330.</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>American Quality Powder Coating; PO 59330; invoice/slip 11055; qty 1, 1, 1, and 3</t>
+          <t>American Quality Powder Coating; PO 59330; packlist 77359; ship date 9/30/2026; qty 1, 1, 1, and 3; no invoice number printed</t>
         </is>
       </c>
     </row>
@@ -812,12 +812,12 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>11058</t>
+          <t>77362</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>20 of 5001914-003 (packlist 77362)</t>
+          <t>20 of 5001914-003</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -828,12 +828,12 @@
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: AQPC invoice 11058, PO 59333, qty 20. No AQPC bill with that invoice or PO.</t>
+          <t>No matching bill yet. Kannon packlist 77362, ship date 9/30/2026, PO 59333, qty 20. No Invoice no. is printed. No AQPC bill on PO 59333.</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>American Quality Powder Coating; PO 59333; invoice/slip 11058; qty 20</t>
+          <t>American Quality Powder Coating; PO 59333; packlist 77362; ship date 9/30/2026; qty 20 of 5001914-003; no invoice number printed</t>
         </is>
       </c>
     </row>
@@ -870,7 +870,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>48 of KANNON-ME26-1951</t>
+          <t>48 shipped of KANNON-ME26-1951 (ordered 48)</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -881,12 +881,12 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: Legacy Wire shipment S-SHPT103393, order S-ORD102051, PO 59322, qty 48. No Legacy Wire bill on that PO.</t>
+          <t>No matching bill yet. Crop read: shipment S-SHPT103393, order S-ORD102051, date 10/1/2026, PO 59322, qty 48. No Legacy Wire bill on that PO.</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Legacy Wire Products; PO 59322; invoice/slip S-SHPT103393 / S-ORD102051; qty 48</t>
+          <t>Legacy Wire Products; PO 59322; shipment S-SHPT103393; order S-ORD102051; date 10/1/2026; qty 48</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>27 of KANNON-ME26-1951</t>
+          <t>27 shipped of KANNON-ME26-1951 (ordered 27)</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -934,12 +934,12 @@
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: Legacy Wire shipment S-SHPT103392, order S-ORD102050, PO 59334, qty 27. No Legacy Wire bill on that PO.</t>
+          <t>No matching bill yet. Crop read: shipment S-SHPT103392, order S-ORD102050, date 10/1/2026, PO 59334, qty 27. No Legacy Wire bill on that PO.</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Legacy Wire Products; PO 59334; invoice/slip S-SHPT103392 / S-ORD102050; qty 27</t>
+          <t>Legacy Wire Products; PO 59334; shipment S-SHPT103392; order S-ORD102050; date 10/1/2026; qty 27</t>
         </is>
       </c>
     </row>
@@ -983,12 +983,12 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Not a packing slip. Eye read is a Kannon purchase order 59337 to JARTEX, qty required 90. Left off.</t>
+          <t>Not a packing slip. Crop read is Kannon purchase order 59337 to JARTEX, date 9/30/2026, qty required 90. Left off.</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>JARTEX Industries (purchase order, not a packing slip); PO 59337; invoice/slip —; qty 90 ordered</t>
+          <t>JARTEX Industries (purchase order, not a packing slip); PO 59337; date 9/30/2026; qty 90 ordered</t>
         </is>
       </c>
     </row>
@@ -1015,17 +1015,17 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>59331</t>
+          <t>59321</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>11056</t>
+          <t>11055</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>1 each of A060R267, A059J397, 70040164, A059J396</t>
+          <t>1 each of AMT-A060R267, AMT-A059J397, AMT-70040164, AMT-A059J396</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -1036,12 +1036,12 @@
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: AQPC invoice 11056, PO 59331, qty 1 each. The formal packlist for the same invoice shows A059J397 qty 4. No AQPC bill to attach to either page.</t>
+          <t>No matching bill yet. Header crop: Invoice no. 11055, date 10/01/2026, P.O. Number 59321, qty 1 on each of four lines. No AQPC bill with invoice 11055 or PO 59321.</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>American Quality Powder Coating; PO 59331; invoice/slip 11056; qty 1, 1, 1, 1</t>
+          <t>American Quality Powder Coating; PO 59321; invoice 11055; date 10/01/2026; qty 1, 1, 1, 1</t>
         </is>
       </c>
     </row>
@@ -1068,12 +1068,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>59330</t>
+          <t>59339</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>11055</t>
+          <t>11056</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1089,12 +1089,12 @@
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: AQPC invoice 11055, PO 59330, qty 3 and 3. Consistent with the itemized packlist (1+1+1 and 3). No AQPC bill with that invoice or PO.</t>
+          <t>No matching bill yet. Header crop: Invoice no. 11056, date 10/01/2026, P.O. Number 59339, qty 3 and 3. No AQPC bill with invoice 11056 or PO 59339.</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>American Quality Powder Coating; PO 59330; invoice/slip 11055; qty 3 and 3</t>
+          <t>American Quality Powder Coating; PO 59339; invoice 11056; date 10/01/2026; qty 3 and 3</t>
         </is>
       </c>
     </row>
@@ -1126,12 +1126,12 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>6-175802</t>
+          <t>77391</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>6 of 12519-2 (packlist 77391)</t>
+          <t>6 of 12519-2</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
@@ -1142,12 +1142,12 @@
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: Arrow invoice 6-175802, PO 59321, qty 6. No Arrow bill with that invoice or PO.</t>
+          <t>No matching bill yet. Kannon packlist 77391 to Arrow Plating, ship date 9/30/2026, PO 59321, qty 6. No Arrow invoice number is printed on this page. No Arrow bill on PO 59321.</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Arrow Plating; PO 59321; invoice/slip 6-175802; qty 6 of 12519-2</t>
+          <t>Arrow Plating; PO 59321; packlist 77391; ship date 9/30/2026; qty 6 of 12519-2; no Arrow invoice number printed</t>
         </is>
       </c>
     </row>
@@ -1195,12 +1195,12 @@
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: Crosslink slip 5493, PO 59258, qty 1 and 2. No Crosslink bill for that slip or PO.</t>
+          <t>No matching bill yet. Crosslink slip 5493, date Wed Sep 30 2026, PO 59258, qty 1 and 2. No Crosslink bill for that slip or PO.</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Crosslink Powder Coating; PO 59258; invoice/slip 5493; qty 1 and 2</t>
+          <t>Crosslink Powder Coating; PO 59258; slip 5493; date Sep 30, 2026; qty 1 of 1020249-1 and 2 of 1020249-4</t>
         </is>
       </c>
     </row>
@@ -1248,12 +1248,12 @@
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: AQPC invoice 11053, PO 59311, date 09/30/2026, qty 12. No AQPC bill with invoice 11053 or PO 59311. KANNON/CDM invoice 59311 (id 1298) is a different vendor.</t>
+          <t>No matching bill yet. Header crop: Invoice no. 11053, date 09/30/2026, P.O. Number 59311, qty 12. No AQPC bill with invoice 11053 or PO 59311. KANNON/CDM invoice 59311 (id 1298) is a different vendor.</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>American Quality Powder Coating; PO 59311; invoice/slip 11053; qty 12 of AMT-F1508</t>
+          <t>American Quality Powder Coating; PO 59311; invoice 11053; date 09/30/2026; qty 12 of AMT-F1508</t>
         </is>
       </c>
     </row>
@@ -1290,7 +1290,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>15 of A060P934</t>
+          <t>15 of AMT-A060P934</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -1301,12 +1301,12 @@
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: AQPC invoice 11052, PO 59315, qty 15. No AQPC bill with that invoice or PO.</t>
+          <t>No matching bill yet. Header crop: Invoice no. 11052, date 09/30/2026, P.O. Number 59315, qty 15. No AQPC bill with that invoice or PO.</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>American Quality Powder Coating; PO 59315; invoice/slip 11052; qty 15 of A060P934</t>
+          <t>American Quality Powder Coating; PO 59315; invoice 11052; date 09/30/2026; qty 15 of AMT-A060P934</t>
         </is>
       </c>
     </row>
@@ -1338,12 +1338,12 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>11050</t>
+          <t>11051</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>5 of 5003557-001</t>
+          <t>5 of AMT-5003557-001</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -1354,12 +1354,12 @@
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: AQPC invoice 11050, PO 59312, qty 5. No AQPC bill with that invoice or PO.</t>
+          <t>No matching bill yet. Header crop: Invoice no. 11051, date 09/30/2026, P.O. Number 59312, qty 5. No AQPC bill with that invoice or PO.</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>American Quality Powder Coating; PO 59312; invoice/slip 11050; qty 5 of 5003557-001</t>
+          <t>American Quality Powder Coating; PO 59312; invoice 11051; date 09/30/2026; qty 5 of AMT-5003557-001</t>
         </is>
       </c>
     </row>
@@ -1391,12 +1391,12 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>11049</t>
+          <t>11050</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>10 of 5003557-001</t>
+          <t>10 of AMT-5003557-001</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
@@ -1407,12 +1407,12 @@
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: AQPC invoice 11049, PO 59314, qty 10. No AQPC bill with that invoice or PO.</t>
+          <t>No matching bill yet. Header crop: Invoice no. 11050, date 09/30/2026, P.O. Number 59314, qty 10. No AQPC bill with that invoice or PO.</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>American Quality Powder Coating; PO 59314; invoice/slip 11049; qty 10 of 5003557-001</t>
+          <t>American Quality Powder Coating; PO 59314; invoice 11050; date 09/30/2026; qty 10 of AMT-5003557-001</t>
         </is>
       </c>
     </row>
@@ -1439,17 +1439,17 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>59313</t>
+          <t>59281</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>11051</t>
+          <t>11049</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>12 of 55700014</t>
+          <t>12 of AMT-55700014</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
@@ -1460,12 +1460,12 @@
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: AQPC invoice 11051, PO 59313, qty 12. No AQPC bill with that invoice or PO.</t>
+          <t>No matching bill yet. Header crop: Invoice no. 11049, date 09/30/2026, P.O. Number 59281, qty 12. No AQPC bill with that invoice or PO.</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>American Quality Powder Coating; PO 59313; invoice/slip 11051; qty 12 of 55700014</t>
+          <t>American Quality Powder Coating; PO 59281; invoice 11049; date 09/30/2026; qty 12 of AMT-55700014</t>
         </is>
       </c>
     </row>
@@ -1497,12 +1497,12 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>11048</t>
+          <t>11047</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>18 of A074A683; 18 of A074A682; 10 of 5001914; 1 of 80341994</t>
+          <t>18 of AMT-A074A683; 18 of AMT-A074A682; 10 of AMT-5001914; 1 of AMT-80341994</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -1513,12 +1513,12 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: AQPC invoice 11048, PO 59298, those four quantities. No AQPC bill with that invoice or PO.</t>
+          <t>No matching bill yet. Header crop: Invoice no. 11047, date 09/30/2026, P.O. Number 59298, those four quantities. No AQPC bill with that invoice or PO.</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>American Quality Powder Coating; PO 59298; invoice/slip 11048; qty 18, 18, 10, 1</t>
+          <t>American Quality Powder Coating; PO 59298; invoice 11047; date 09/30/2026; qty 18, 18, 10, 1</t>
         </is>
       </c>
     </row>
@@ -1566,12 +1566,12 @@
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: Crosslink slip 5499, PO 59225, qty 1. No Crosslink bill for that slip or PO.</t>
+          <t>No matching bill yet. Crosslink slip 5499, date Wed Sep 30 2026, PO 59225, qty 1. No Crosslink bill for that slip or PO. KANNON/CDM invoice 59225 (id 1291) is a different vendor.</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Crosslink Powder Coating; PO 59225; invoice/slip 5499; qty 1 of 1020249-1</t>
+          <t>Crosslink Powder Coating; PO 59225; slip 5499; date Sep 30, 2026; qty 1 of 1020249-1</t>
         </is>
       </c>
     </row>
@@ -1619,12 +1619,12 @@
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: Arrow order 179924, PO 58743, qty 350. No Arrow bill on that PO.</t>
+          <t>No matching bill yet. Arrow shipping ticket, order 179924, ship date 9/30/2026, PO 58743, qty 350. No Arrow bill on that PO.</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Arrow Plating; PO 58743; invoice/slip 179924; qty 350 of 1007092-1</t>
+          <t>Arrow Plating; PO 58743; order 179924; ship date 9/30/2026; qty 350 of 1007092-1</t>
         </is>
       </c>
     </row>
@@ -1651,17 +1651,17 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>59302</t>
+          <t>59276</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>11041</t>
+          <t>11042</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>5, 5, 5, 15, 5, 5 (SO34645 basket set)</t>
+          <t>5 of AMT-6001232; 5 of AMT-5003753; 5 of AMT-5003753; 15 of AMT-5003741; 5 of AMT-5003750-002; 5 of AMT-5003750</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
@@ -1672,12 +1672,12 @@
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: AQPC invoice 11041, PO 59302. No AQPC bill with that invoice or PO.</t>
+          <t>No matching bill yet. Header crop: Invoice no. 11042, date 09/29/2026, P.O. Number 59276, those six quantities. No AQPC bill with invoice 11042 or PO 59276. KANNON/CDM invoice 59276 (id 284) is a different vendor.</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>American Quality Powder Coating; PO 59302; invoice/slip 11041; qty 5, 5, 5, 15, 5, 5</t>
+          <t>American Quality Powder Coating; PO 59276; invoice 11042; date 09/29/2026; qty 5, 5, 5, 15, 5, 5</t>
         </is>
       </c>
     </row>
@@ -1704,17 +1704,17 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>59287</t>
+          <t>59283</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>11042</t>
+          <t>11043</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>5 of 5003522-001</t>
+          <t>5 of AMT-5003522-001</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
@@ -1725,12 +1725,12 @@
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: AQPC invoice 11042, PO 59287, qty 5. No AQPC bill with that invoice or PO.</t>
+          <t>No matching bill yet. Header crop: Invoice no. 11043, date 09/29/2026, P.O. Number 59283, qty 5. No AQPC bill with that invoice or PO.</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>American Quality Powder Coating; PO 59287; invoice/slip 11042; qty 5 of 5003522-001</t>
+          <t>American Quality Powder Coating; PO 59283; invoice 11043; date 09/29/2026; qty 5 of AMT-5003522-001</t>
         </is>
       </c>
     </row>
@@ -1757,17 +1757,17 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>59303</t>
+          <t>59171</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>11043</t>
+          <t>11044</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>1, 1, 1, 3, 1, 1 (P089476 basket set)</t>
+          <t>1 of AMT-6001232; 1 of AMT-5003753; 1 of AMT-5003753; 3 of AMT-5003741; 1 of AMT-5003750-002; 1 of AMT-5003750</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
@@ -1778,12 +1778,12 @@
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: AQPC invoice 11043, PO 59303. No AQPC bill with that invoice or PO.</t>
+          <t>No matching bill yet. Header crop: Invoice no. 11044, date 09/29/2026, P.O. Number 59171, those six quantities. No AQPC bill with that invoice or PO.</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>American Quality Powder Coating; PO 59303; invoice/slip 11043; qty 1, 1, 1, 3, 1, 1</t>
+          <t>American Quality Powder Coating; PO 59171; invoice 11044; date 09/29/2026; qty 1, 1, 1, 3, 1, 1</t>
         </is>
       </c>
     </row>
@@ -1815,7 +1815,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>11044</t>
+          <t>11041</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -1831,12 +1831,12 @@
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: AQPC invoice 11044, PO 59274, qty 250. No AQPC bill with invoice 11044 or PO 59274. A different slip (invoice 11054, packlist 77271) is also qty 250 on PO 59274.</t>
+          <t>No matching bill yet. Header crop: Invoice no. 11041, date 09/28/2026, P.O. Number 59274, qty 250. No AQPC bill with invoice 11041 or PO 59274. KANNON/CDM invoice 59274 (id 286) is a different vendor.</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>American Quality Powder Coating; PO 59274; invoice/slip 11044; qty 250 of KAN-MD04</t>
+          <t>American Quality Powder Coating; PO 59274; invoice 11041; date 09/28/2026; qty 250 of KAN-MD04</t>
         </is>
       </c>
     </row>
@@ -1868,12 +1868,12 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>6-175800</t>
+          <t>77329</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>26 of 5003004-001 (packlist 77329)</t>
+          <t>26 of 5003004-001</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
@@ -1884,12 +1884,12 @@
       <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: Arrow invoice 6-175800, PO 59310, qty 26. No Arrow bill with that invoice or PO.</t>
+          <t>No matching bill yet. Kannon packlist 77329 to Arrow, ship date 9/29/2026, PO 59310, qty 26. No Arrow invoice number is printed. No Arrow bill on PO 59310.</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>Arrow Plating; PO 59310; invoice/slip 6-175800; qty 26 of 5003004-001</t>
+          <t>Arrow Plating; PO 59310; packlist 77329; ship date 9/29/2026; qty 26 of 5003004-001</t>
         </is>
       </c>
     </row>
@@ -1921,12 +1921,12 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>6-175797</t>
+          <t>77326</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>2 of 33214-1 (packlist 77326)</t>
+          <t>2 of 33214-1</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
@@ -1937,12 +1937,12 @@
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: Arrow invoice 6-175797, PO 59307, qty 2. No Arrow bill with that invoice or PO.</t>
+          <t>No matching bill yet. Kannon packlist 77326 to Arrow, ship date 9/29/2026, PO 59307, qty 2. No Arrow invoice number is printed. No Arrow bill on PO 59307.</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>Arrow Plating; PO 59307; invoice/slip 6-175797; qty 2 of 33214-1</t>
+          <t>Arrow Plating; PO 59307; packlist 77326; ship date 9/29/2026; qty 2 of 33214-1</t>
         </is>
       </c>
     </row>
@@ -1974,12 +1974,12 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>6-175799</t>
+          <t>77328</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>100 of 7766-1 (packlist 77328)</t>
+          <t>100 of 7766-1</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
@@ -1990,12 +1990,12 @@
       <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: Arrow invoice 6-175799, PO 59309, qty 100. No Arrow bill with that invoice or PO.</t>
+          <t>No matching bill yet. Kannon packlist 77328 to Arrow, ship date 9/29/2026, PO 59309, qty 100. No Arrow invoice number is printed. No Arrow bill on PO 59309. KANNON/CDM invoice 59309 (id 1297) is a different vendor.</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>Arrow Plating; PO 59309; invoice/slip 6-175799; qty 100 of 7766-1</t>
+          <t>Arrow Plating; PO 59309; packlist 77328; ship date 9/29/2026; qty 100 of 7766-1</t>
         </is>
       </c>
     </row>
@@ -2027,12 +2027,12 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>6-175798</t>
+          <t>77327</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>300 of 7766-1 (packlist 77327)</t>
+          <t>300 of 7766-1</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
@@ -2043,12 +2043,12 @@
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: Arrow invoice 6-175798, PO 59308, qty 300. No Arrow bill with that invoice or PO.</t>
+          <t>No matching bill yet. Kannon packlist 77327 to Arrow, ship date 9/29/2026, PO 59308, qty 300. No Arrow invoice number is printed. No Arrow bill on PO 59308.</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>Arrow Plating; PO 59308; invoice/slip 6-175798; qty 300 of 7766-1</t>
+          <t>Arrow Plating; PO 59308; packlist 77327; ship date 9/29/2026; qty 300 of 7766-1</t>
         </is>
       </c>
     </row>
@@ -2080,12 +2080,12 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>11049</t>
+          <t>77332</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>10 of 5003557-001 (packlist 77332)</t>
+          <t>10 of 5003557-001</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
@@ -2096,12 +2096,12 @@
       <c r="I31" s="2" t="inlineStr"/>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: AQPC invoice 11049, PO 59314, qty 10. Same invoice as the letterhead page. No AQPC bill with that invoice or PO.</t>
+          <t>No matching bill yet. Kannon packlist 77332, ship date 9/29/2026, PO 59314, qty 10. No Invoice no. is printed. No AQPC bill on PO 59314.</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>American Quality Powder Coating; PO 59314; invoice/slip 11049; qty 10 of 5003557-001</t>
+          <t>American Quality Powder Coating; PO 59314; packlist 77332; ship date 9/29/2026; qty 10 of 5003557-001; no invoice number printed</t>
         </is>
       </c>
     </row>
@@ -2133,12 +2133,12 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>11050</t>
+          <t>77331</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>5 of 5003557-001 (packlist 77331)</t>
+          <t>5 of 5003557-001</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
@@ -2149,12 +2149,12 @@
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: AQPC invoice 11050, PO 59312, qty 5. Same invoice as the letterhead page. No AQPC bill with that invoice or PO.</t>
+          <t>No matching bill yet. Kannon packlist 77331, ship date 9/29/2026, PO 59312, qty 5. No Invoice no. is printed. No AQPC bill on PO 59312.</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>American Quality Powder Coating; PO 59312; invoice/slip 11050; qty 5 of 5003557-001</t>
+          <t>American Quality Powder Coating; PO 59312; packlist 77331; ship date 9/29/2026; qty 5 of 5003557-001; no invoice number printed</t>
         </is>
       </c>
     </row>
@@ -2186,12 +2186,12 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>11052</t>
+          <t>77333</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>15 of A060P934 (packlist 77333)</t>
+          <t>15 of A060P934</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -2202,12 +2202,12 @@
       <c r="I33" s="2" t="inlineStr"/>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: AQPC invoice 11052, PO 59315, qty 15. Same invoice as the letterhead page. No AQPC bill with that invoice or PO.</t>
+          <t>No matching bill yet. Kannon packlist 77333, ship date 9/29/2026, PO 59315, qty 15. No Invoice no. is printed. No AQPC bill on PO 59315.</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>American Quality Powder Coating; PO 59315; invoice/slip 11052; qty 15 of A060P934</t>
+          <t>American Quality Powder Coating; PO 59315; packlist 77333; ship date 9/29/2026; qty 15 of A060P934; no invoice number printed</t>
         </is>
       </c>
     </row>
@@ -2239,12 +2239,12 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>11053</t>
+          <t>77330</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>12 of F1508 (packlist 77330)</t>
+          <t>12 of F1508</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
@@ -2255,12 +2255,12 @@
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: AQPC invoice 11053, PO 59311, qty 12. Same invoice Kyle checked on the letterhead page. No AQPC bill with invoice 11053 or PO 59311.</t>
+          <t>No matching bill yet. Kannon packlist 77330, ship date 9/29/2026, PO 59311, qty 12 of F1508. No Invoice no. is printed. No AQPC bill on PO 59311.</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>American Quality Powder Coating; PO 59311; invoice/slip 11053; qty 12 of F1508</t>
+          <t>American Quality Powder Coating; PO 59311; packlist 77330; ship date 9/29/2026; qty 12 of F1508; no invoice number printed</t>
         </is>
       </c>
     </row>
@@ -2292,12 +2292,12 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>11048</t>
+          <t>77311</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>18, 18, 10, 1 (packlist 77341)</t>
+          <t>18 of A074A683; 18 of A074A682; 10 of 5001914-003; 1 of 80341994</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
@@ -2308,12 +2308,12 @@
       <c r="I35" s="2" t="inlineStr"/>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: AQPC invoice 11048, PO 59298, qty 18, 18, 10, and 1. Same invoice as the letterhead page. No AQPC bill with that invoice or PO.</t>
+          <t>No matching bill yet. Kannon packlist 77311, ship date 9/28/2026, PO 59298, qty 18, 18, 10, and 1. No Invoice no. is printed. No AQPC bill on PO 59298.</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>American Quality Powder Coating; PO 59298; invoice/slip 11048; qty 18, 18, 10, 1</t>
+          <t>American Quality Powder Coating; PO 59298; packlist 77311; ship date 9/28/2026; qty 18, 18, 10, 1; no invoice number printed</t>
         </is>
       </c>
     </row>
@@ -2361,12 +2361,12 @@
       <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: Arrow order 179880, PO 58722, qty 100. No Arrow bill on that PO.</t>
+          <t>No matching bill yet. Arrow shipping ticket, order 179880, ship date 9/23/2026, PO 58722, qty 100. No Arrow bill on that PO.</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>Arrow Plating; PO 58722; invoice/slip 179880; qty 100 of 11772-1</t>
+          <t>Arrow Plating; PO 58722; order 179880; ship date 9/23/2026; qty 100 of 11772-1</t>
         </is>
       </c>
     </row>
@@ -2414,12 +2414,12 @@
       <c r="I37" s="2" t="inlineStr"/>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: Arrow order 180005, PO 58882, qty 50. No Arrow bill on that PO.</t>
+          <t>No matching bill yet. Arrow shipping ticket, order 180005, ship date 9/23/2026, PO 58882, qty 50. No Arrow bill on that PO.</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>Arrow Plating; PO 58882; invoice/slip 180005; qty 50 of 11772-1</t>
+          <t>Arrow Plating; PO 58882; order 180005; ship date 9/23/2026; qty 50 of 11772-1</t>
         </is>
       </c>
     </row>
@@ -2451,12 +2451,12 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>11054</t>
+          <t>77271</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>250 of MD04-1661 (packlist 77271, marked page 4)</t>
+          <t>250 of MD04-1661</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
@@ -2467,12 +2467,12 @@
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: AQPC invoice 11054, PO 59274, qty 250. No AQPC bill with invoice 11054 or PO 59274.</t>
+          <t>No matching bill yet. Kannon packlist 77271, marked page 4, ship date 9/24/2026, PO 59274, qty 250. No Invoice no. is printed. No AQPC bill on PO 59274.</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>American Quality Powder Coating; PO 59274; invoice/slip 11054; qty 250 of MD04-1661</t>
+          <t>American Quality Powder Coating; PO 59274; packlist 77271 page 4; ship date 9/24/2026; qty 250 of MD04-1661; no invoice number printed</t>
         </is>
       </c>
     </row>
@@ -2525,7 +2525,7 @@
       <c r="J39" s="2" t="inlineStr"/>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>McMaster-Carr; PO 59235; invoice/slip 5756929-01; qty ordered 3, shipped 3 of 91306A416</t>
+          <t>McMaster-Carr; PO 59235; packing list 5756929-01; ordered 3, shipped 3 of 91306A416</t>
         </is>
       </c>
     </row>
@@ -2573,12 +2573,12 @@
       <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: McMaster PO 58221, qty 24. The only live bill on PO 58221 is AQPC invoice 10655 (id 8827). Vendor does not match.</t>
+          <t>No matching bill yet. Crop read: McMaster PO 58221, list 5687917-01, ordered 24, shipped 24. The only live bill on PO 58221 is AQPC invoice 10655 (id 8827). Vendor does not match.</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>McMaster-Carr; PO 58221; invoice/slip 5687917-01; qty ordered 24, shipped 24 of 4082715</t>
+          <t>McMaster-Carr; PO 58221; packing list 5687917-01; ordered 24, shipped 24 of 4082715</t>
         </is>
       </c>
     </row>
@@ -2631,7 +2631,7 @@
       <c r="J41" s="2" t="inlineStr"/>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>McMaster-Carr; PO 59191; invoice/slip 5539373-01; qty ordered 40, shipped 40 of 91247A860</t>
+          <t>McMaster-Carr; PO 59191; packing list 5539373-01; ordered 40, shipped 40 of 91247A860</t>
         </is>
       </c>
     </row>
@@ -2668,7 +2668,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>line 4 shipped 1 of 93320A385 (ordered 2); lines 1-3 also printed</t>
+          <t>line 4 shipped 1 of 93320A385 (ordered 2); lines 1-3 shipped 6, 1, and 1</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
@@ -2684,7 +2684,7 @@
       <c r="J42" s="2" t="inlineStr"/>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>McMaster-Carr; PO 59224; invoice/slip 5765761-01; qty line 4 ordered 2, shipped 1</t>
+          <t>McMaster-Carr; PO 59224; packing list 5765761-01; line 4 ordered 2, shipped 1; lines 1-3 shipped 6, 1, 1</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2721,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>line 4 shipped 1 of 93320A385; lines 1-3 shipped 6, 1, and 1</t>
+          <t>line 4 shipped 1 of 93320A385 (ordered 2); lines 1-3 shipped 6, 1, and 1</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
@@ -2732,12 +2732,12 @@
       <c r="I43" s="2" t="inlineStr"/>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>Qty conflict. Eye read: McMaster list 5765761-02, PO 59224, line 4 shipped 1. Bill 10142 is PO line 04 qty 1 and already has list 5765761-01 (also line 4 shipped 1). Putting this second shipment on that bill would show shipped qty 2 against qty 1. Left off. A prior file packing-slip-59224-page 2.pdf is already on the bill and was not removed.</t>
+          <t>Qty conflict. Crop read: McMaster list 5765761-02, PO 59224, line 4 shipped 1. Bill 10142 is PO line 04 qty 1 and already has list 5765761-01 (also line 4 shipped 1). Putting this second shipment on that bill would show shipped qty 2 against qty 1. Left off. A prior file packing-slip-59224-page 2.pdf is already on the bill and was not removed.</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>McMaster-Carr; PO 59224; invoice/slip 5765761-02; qty line 4 ordered 2, shipped 1; lines 1-3 shipped 6, 1, 1</t>
+          <t>McMaster-Carr; PO 59224; packing list 5765761-02; line 4 ordered 2, shipped 1; lines 1-3 shipped 6, 1, 1</t>
         </is>
       </c>
     </row>
@@ -2785,12 +2785,12 @@
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>No matching bill yet. Eye read: McMaster PO 59149, order 5680403-07, qty 40 of 91247A866. No McMaster bill on PO 59149.</t>
+          <t>No matching bill yet. Crop read: McMaster PO 59149, list 5680403-07, ordered 40, shipped 40 of 91247A866. No McMaster bill on PO 59149.</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>McMaster-Carr; PO 59149; invoice/slip 5680403-07; qty ordered 40, shipped 40 of 91247A866</t>
+          <t>McMaster-Carr; PO 59149; packing list 5680403-07; ordered 40, shipped 40 of 91247A866</t>
         </is>
       </c>
     </row>

</xml_diff>